<commit_message>
Modificaciones de estos archivos en la parte de consultas, las consultas que estaban en el jsp se pasaron al administrador de consultas, algunos archivos no tenian consultas.
</commit_message>
<xml_diff>
--- a/Control.xlsx
+++ b/Control.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\sigma_pruebas1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\10.106.12.32\compartir\openlayers2_nvo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDA29665-E921-4F16-A735-ADF6D91C79BF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{526BABFF-BB27-4798-BE81-221A2BF88BC2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="13905" xr2:uid="{119285BF-BAF3-43BB-BF3D-96AE8CA3F258}"/>
   </bookViews>
@@ -432,9 +432,6 @@
     <t>amapa.html</t>
   </si>
   <si>
-    <t>astyle.css</t>
-  </si>
-  <si>
     <t>avance_act_mg.html</t>
   </si>
   <si>
@@ -652,6 +649,9 @@
   </si>
   <si>
     <t>zedit-passSigma.jsp</t>
+  </si>
+  <si>
+    <t>Ricardo</t>
   </si>
 </sst>
 </file>
@@ -736,7 +736,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -754,6 +754,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1071,10 +1074,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8CFB12C-C000-4D62-A088-E6A986C2EDDD}">
-  <dimension ref="B1:G204"/>
+  <dimension ref="B1:G208"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="26.7109375" customWidth="1"/>
+    <col min="2" max="2" width="42.140625" customWidth="1"/>
     <col min="3" max="3" width="23.42578125" customWidth="1"/>
     <col min="4" max="4" width="22.85546875" customWidth="1"/>
     <col min="5" max="5" width="24.5703125" customWidth="1"/>
@@ -1105,7 +1108,10 @@
       <c r="B2" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="D2" s="4"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="5" t="s">
+        <v>208</v>
+      </c>
       <c r="E2" s="7"/>
       <c r="F2" s="6"/>
       <c r="G2" s="2"/>
@@ -1168,7 +1174,7 @@
     </row>
     <row r="10" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="4" t="s">
-        <v>135</v>
+        <v>4</v>
       </c>
       <c r="C10" s="4"/>
       <c r="D10" s="5"/>
@@ -1176,7 +1182,7 @@
     </row>
     <row r="11" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C11" s="4"/>
       <c r="D11" s="5"/>
@@ -1184,7 +1190,7 @@
     </row>
     <row r="12" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C12" s="4"/>
       <c r="D12" s="5"/>
@@ -1192,7 +1198,7 @@
     </row>
     <row r="13" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C13" s="4"/>
       <c r="D13" s="5"/>
@@ -1200,7 +1206,7 @@
     </row>
     <row r="14" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C14" s="4"/>
       <c r="D14" s="5"/>
@@ -1208,7 +1214,7 @@
     </row>
     <row r="15" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C15" s="4"/>
       <c r="D15" s="5"/>
@@ -1216,7 +1222,7 @@
     </row>
     <row r="16" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C16" s="4"/>
       <c r="D16" s="5"/>
@@ -1224,7 +1230,7 @@
     </row>
     <row r="17" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="4" t="s">
-        <v>10</v>
+        <v>135</v>
       </c>
       <c r="C17" s="4"/>
       <c r="D17" s="5"/>
@@ -1232,7 +1238,7 @@
     </row>
     <row r="18" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="4" t="s">
-        <v>136</v>
+        <v>11</v>
       </c>
       <c r="C18" s="4"/>
       <c r="D18" s="5"/>
@@ -1240,7 +1246,7 @@
     </row>
     <row r="19" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C19" s="4"/>
       <c r="D19" s="5"/>
@@ -1248,7 +1254,7 @@
     </row>
     <row r="20" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C20" s="4"/>
       <c r="D20" s="5"/>
@@ -1256,7 +1262,7 @@
     </row>
     <row r="21" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C21" s="4"/>
       <c r="D21" s="5"/>
@@ -1264,7 +1270,7 @@
     </row>
     <row r="22" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="4" t="s">
-        <v>14</v>
+        <v>136</v>
       </c>
       <c r="C22" s="4"/>
       <c r="D22" s="5"/>
@@ -1272,7 +1278,7 @@
     </row>
     <row r="23" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="4" t="s">
-        <v>137</v>
+        <v>15</v>
       </c>
       <c r="C23" s="4"/>
       <c r="D23" s="5"/>
@@ -1280,7 +1286,7 @@
     </row>
     <row r="24" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C24" s="4"/>
       <c r="D24" s="5"/>
@@ -1288,7 +1294,7 @@
     </row>
     <row r="25" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C25" s="4"/>
       <c r="D25" s="5"/>
@@ -1296,7 +1302,7 @@
     </row>
     <row r="26" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="4" t="s">
-        <v>17</v>
+        <v>137</v>
       </c>
       <c r="C26" s="4"/>
       <c r="D26" s="5"/>
@@ -1312,7 +1318,7 @@
     </row>
     <row r="28" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="4" t="s">
-        <v>139</v>
+        <v>18</v>
       </c>
       <c r="C28" s="4"/>
       <c r="D28" s="5"/>
@@ -1320,7 +1326,7 @@
     </row>
     <row r="29" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C29" s="4"/>
       <c r="D29" s="5"/>
@@ -1328,7 +1334,7 @@
     </row>
     <row r="30" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="4" t="s">
-        <v>19</v>
+        <v>139</v>
       </c>
       <c r="C30" s="4"/>
       <c r="D30" s="5"/>
@@ -1368,7 +1374,7 @@
     </row>
     <row r="35" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B35" s="4" t="s">
-        <v>144</v>
+        <v>20</v>
       </c>
       <c r="C35" s="4"/>
       <c r="D35" s="5"/>
@@ -1376,7 +1382,7 @@
     </row>
     <row r="36" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C36" s="4"/>
       <c r="D36" s="5"/>
@@ -1384,7 +1390,7 @@
     </row>
     <row r="37" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C37" s="4"/>
       <c r="D37" s="5"/>
@@ -1392,7 +1398,7 @@
     </row>
     <row r="38" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="4" t="s">
-        <v>22</v>
+        <v>144</v>
       </c>
       <c r="C38" s="4"/>
       <c r="D38" s="5"/>
@@ -1424,7 +1430,7 @@
     </row>
     <row r="42" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B42" s="4" t="s">
-        <v>148</v>
+        <v>23</v>
       </c>
       <c r="C42" s="4"/>
       <c r="D42" s="5"/>
@@ -1432,7 +1438,7 @@
     </row>
     <row r="43" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B43" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C43" s="4"/>
       <c r="D43" s="5"/>
@@ -1440,7 +1446,7 @@
     </row>
     <row r="44" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B44" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C44" s="4"/>
       <c r="D44" s="5"/>
@@ -1448,7 +1454,7 @@
     </row>
     <row r="45" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C45" s="4"/>
       <c r="D45" s="5"/>
@@ -1456,7 +1462,7 @@
     </row>
     <row r="46" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B46" s="4" t="s">
-        <v>26</v>
+        <v>148</v>
       </c>
       <c r="C46" s="4"/>
       <c r="D46" s="5"/>
@@ -1464,7 +1470,7 @@
     </row>
     <row r="47" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B47" s="4" t="s">
-        <v>149</v>
+        <v>27</v>
       </c>
       <c r="C47" s="4"/>
       <c r="D47" s="5"/>
@@ -1472,7 +1478,7 @@
     </row>
     <row r="48" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B48" s="4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C48" s="4"/>
       <c r="D48" s="5"/>
@@ -1480,7 +1486,7 @@
     </row>
     <row r="49" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B49" s="4" t="s">
-        <v>28</v>
+        <v>149</v>
       </c>
       <c r="C49" s="4"/>
       <c r="D49" s="5"/>
@@ -1536,15 +1542,15 @@
     </row>
     <row r="56" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B56" s="4" t="s">
-        <v>156</v>
+        <v>29</v>
       </c>
       <c r="C56" s="4"/>
       <c r="D56" s="5"/>
       <c r="E56" s="7"/>
     </row>
     <row r="57" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B57" s="4" t="s">
-        <v>29</v>
+      <c r="B57" s="8" t="s">
+        <v>156</v>
       </c>
       <c r="C57" s="4"/>
       <c r="D57" s="5"/>
@@ -1560,7 +1566,7 @@
     </row>
     <row r="59" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B59" s="4" t="s">
-        <v>158</v>
+        <v>30</v>
       </c>
       <c r="C59" s="4"/>
       <c r="D59" s="5"/>
@@ -1568,7 +1574,7 @@
     </row>
     <row r="60" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B60" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C60" s="4"/>
       <c r="D60" s="5"/>
@@ -1576,7 +1582,7 @@
     </row>
     <row r="61" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B61" s="4" t="s">
-        <v>31</v>
+        <v>158</v>
       </c>
       <c r="C61" s="4"/>
       <c r="D61" s="5"/>
@@ -1656,7 +1662,7 @@
     </row>
     <row r="71" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B71" s="4" t="s">
-        <v>168</v>
+        <v>32</v>
       </c>
       <c r="C71" s="4"/>
       <c r="D71" s="5"/>
@@ -1664,7 +1670,7 @@
     </row>
     <row r="72" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B72" s="4" t="s">
-        <v>32</v>
+        <v>168</v>
       </c>
       <c r="C72" s="4"/>
       <c r="D72" s="5"/>
@@ -1680,7 +1686,7 @@
     </row>
     <row r="74" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B74" s="4" t="s">
-        <v>170</v>
+        <v>33</v>
       </c>
       <c r="C74" s="4"/>
       <c r="D74" s="5"/>
@@ -1688,7 +1694,7 @@
     </row>
     <row r="75" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B75" s="4" t="s">
-        <v>33</v>
+        <v>170</v>
       </c>
       <c r="C75" s="4"/>
       <c r="D75" s="5"/>
@@ -1704,7 +1710,7 @@
     </row>
     <row r="77" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B77" s="4" t="s">
-        <v>172</v>
+        <v>34</v>
       </c>
       <c r="C77" s="4"/>
       <c r="D77" s="5"/>
@@ -1712,7 +1718,7 @@
     </row>
     <row r="78" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B78" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C78" s="4"/>
       <c r="D78" s="5"/>
@@ -1720,7 +1726,7 @@
     </row>
     <row r="79" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B79" s="4" t="s">
-        <v>35</v>
+        <v>172</v>
       </c>
       <c r="C79" s="4"/>
       <c r="D79" s="5"/>
@@ -1728,7 +1734,7 @@
     </row>
     <row r="80" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B80" s="4" t="s">
-        <v>173</v>
+        <v>36</v>
       </c>
       <c r="C80" s="4"/>
       <c r="D80" s="5"/>
@@ -1736,7 +1742,7 @@
     </row>
     <row r="81" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B81" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C81" s="4"/>
       <c r="D81" s="5"/>
@@ -1744,7 +1750,7 @@
     </row>
     <row r="82" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B82" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C82" s="4"/>
       <c r="D82" s="5"/>
@@ -1752,7 +1758,7 @@
     </row>
     <row r="83" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B83" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C83" s="4"/>
       <c r="D83" s="5"/>
@@ -1760,7 +1766,7 @@
     </row>
     <row r="84" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B84" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C84" s="4"/>
       <c r="D84" s="5"/>
@@ -1768,7 +1774,7 @@
     </row>
     <row r="85" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B85" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C85" s="4"/>
       <c r="D85" s="5"/>
@@ -1776,7 +1782,7 @@
     </row>
     <row r="86" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B86" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C86" s="4"/>
       <c r="D86" s="5"/>
@@ -1784,7 +1790,7 @@
     </row>
     <row r="87" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B87" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C87" s="4"/>
       <c r="D87" s="5"/>
@@ -1792,7 +1798,7 @@
     </row>
     <row r="88" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B88" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C88" s="4"/>
       <c r="D88" s="5"/>
@@ -1800,7 +1806,7 @@
     </row>
     <row r="89" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B89" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C89" s="4"/>
       <c r="D89" s="5"/>
@@ -1808,7 +1814,7 @@
     </row>
     <row r="90" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B90" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C90" s="4"/>
       <c r="D90" s="5"/>
@@ -1816,7 +1822,7 @@
     </row>
     <row r="91" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B91" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C91" s="4"/>
       <c r="D91" s="5"/>
@@ -1824,7 +1830,7 @@
     </row>
     <row r="92" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B92" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C92" s="4"/>
       <c r="D92" s="5"/>
@@ -1832,7 +1838,7 @@
     </row>
     <row r="93" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B93" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C93" s="4"/>
       <c r="D93" s="5"/>
@@ -1840,7 +1846,7 @@
     </row>
     <row r="94" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B94" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C94" s="4"/>
       <c r="D94" s="5"/>
@@ -1848,7 +1854,7 @@
     </row>
     <row r="95" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B95" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C95" s="4"/>
       <c r="D95" s="5"/>
@@ -1856,7 +1862,7 @@
     </row>
     <row r="96" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B96" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C96" s="4"/>
       <c r="D96" s="5"/>
@@ -1864,7 +1870,7 @@
     </row>
     <row r="97" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B97" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C97" s="4"/>
       <c r="D97" s="5"/>
@@ -1872,7 +1878,7 @@
     </row>
     <row r="98" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B98" s="4" t="s">
-        <v>53</v>
+        <v>173</v>
       </c>
       <c r="C98" s="4"/>
       <c r="D98" s="5"/>
@@ -1880,7 +1886,7 @@
     </row>
     <row r="99" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B99" s="4" t="s">
-        <v>174</v>
+        <v>54</v>
       </c>
       <c r="C99" s="4"/>
       <c r="D99" s="5"/>
@@ -1888,7 +1894,7 @@
     </row>
     <row r="100" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B100" s="4" t="s">
-        <v>54</v>
+        <v>174</v>
       </c>
       <c r="C100" s="4"/>
       <c r="D100" s="5"/>
@@ -1896,7 +1902,7 @@
     </row>
     <row r="101" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B101" s="4" t="s">
-        <v>175</v>
+        <v>55</v>
       </c>
       <c r="C101" s="4"/>
       <c r="D101" s="5"/>
@@ -1904,7 +1910,7 @@
     </row>
     <row r="102" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B102" s="4" t="s">
-        <v>55</v>
+        <v>175</v>
       </c>
       <c r="C102" s="4"/>
       <c r="D102" s="5"/>
@@ -1912,7 +1918,7 @@
     </row>
     <row r="103" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B103" s="4" t="s">
-        <v>176</v>
+        <v>56</v>
       </c>
       <c r="C103" s="4"/>
       <c r="D103" s="5"/>
@@ -1920,7 +1926,7 @@
     </row>
     <row r="104" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B104" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C104" s="4"/>
       <c r="D104" s="5"/>
@@ -1928,7 +1934,7 @@
     </row>
     <row r="105" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B105" s="4" t="s">
-        <v>57</v>
+        <v>176</v>
       </c>
       <c r="C105" s="4"/>
       <c r="D105" s="5"/>
@@ -1944,7 +1950,7 @@
     </row>
     <row r="107" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B107" s="4" t="s">
-        <v>178</v>
+        <v>58</v>
       </c>
       <c r="C107" s="4"/>
       <c r="D107" s="5"/>
@@ -1952,7 +1958,7 @@
     </row>
     <row r="108" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B108" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C108" s="4"/>
       <c r="D108" s="5"/>
@@ -1960,7 +1966,7 @@
     </row>
     <row r="109" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B109" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C109" s="4"/>
       <c r="D109" s="5"/>
@@ -1968,7 +1974,7 @@
     </row>
     <row r="110" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B110" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C110" s="4"/>
       <c r="D110" s="5"/>
@@ -1976,7 +1982,7 @@
     </row>
     <row r="111" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B111" s="4" t="s">
-        <v>61</v>
+        <v>178</v>
       </c>
       <c r="C111" s="4"/>
       <c r="D111" s="5"/>
@@ -1984,7 +1990,7 @@
     </row>
     <row r="112" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B112" s="4" t="s">
-        <v>179</v>
+        <v>62</v>
       </c>
       <c r="C112" s="4"/>
       <c r="D112" s="5"/>
@@ -1992,7 +1998,7 @@
     </row>
     <row r="113" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B113" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C113" s="4"/>
       <c r="D113" s="5"/>
@@ -2000,7 +2006,7 @@
     </row>
     <row r="114" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B114" s="4" t="s">
-        <v>63</v>
+        <v>179</v>
       </c>
       <c r="C114" s="4"/>
       <c r="D114" s="5"/>
@@ -2008,7 +2014,7 @@
     </row>
     <row r="115" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B115" s="4" t="s">
-        <v>180</v>
+        <v>64</v>
       </c>
       <c r="C115" s="4"/>
       <c r="D115" s="5"/>
@@ -2016,7 +2022,7 @@
     </row>
     <row r="116" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B116" s="4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C116" s="4"/>
       <c r="D116" s="5"/>
@@ -2024,7 +2030,7 @@
     </row>
     <row r="117" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B117" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C117" s="4"/>
       <c r="D117" s="5"/>
@@ -2032,7 +2038,7 @@
     </row>
     <row r="118" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B118" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C118" s="4"/>
       <c r="D118" s="5"/>
@@ -2040,7 +2046,7 @@
     </row>
     <row r="119" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B119" s="4" t="s">
-        <v>67</v>
+        <v>180</v>
       </c>
       <c r="C119" s="4"/>
       <c r="D119" s="5"/>
@@ -2048,7 +2054,7 @@
     </row>
     <row r="120" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B120" s="4" t="s">
-        <v>181</v>
+        <v>68</v>
       </c>
       <c r="C120" s="4"/>
       <c r="D120" s="5"/>
@@ -2056,7 +2062,7 @@
     </row>
     <row r="121" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B121" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C121" s="4"/>
       <c r="D121" s="5"/>
@@ -2064,7 +2070,7 @@
     </row>
     <row r="122" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B122" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C122" s="4"/>
       <c r="D122" s="5"/>
@@ -2072,7 +2078,7 @@
     </row>
     <row r="123" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B123" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C123" s="4"/>
       <c r="D123" s="5"/>
@@ -2080,7 +2086,7 @@
     </row>
     <row r="124" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B124" s="4" t="s">
-        <v>71</v>
+        <v>181</v>
       </c>
       <c r="C124" s="4"/>
       <c r="D124" s="5"/>
@@ -2088,7 +2094,7 @@
     </row>
     <row r="125" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B125" s="4" t="s">
-        <v>182</v>
+        <v>72</v>
       </c>
       <c r="C125" s="4"/>
       <c r="D125" s="5"/>
@@ -2096,7 +2102,7 @@
     </row>
     <row r="126" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B126" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C126" s="4"/>
       <c r="D126" s="5"/>
@@ -2104,7 +2110,7 @@
     </row>
     <row r="127" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B127" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C127" s="4"/>
       <c r="D127" s="5"/>
@@ -2112,7 +2118,7 @@
     </row>
     <row r="128" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B128" s="4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C128" s="4"/>
       <c r="D128" s="5"/>
@@ -2120,389 +2126,621 @@
     </row>
     <row r="129" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B129" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C129" s="4"/>
       <c r="D129" s="5"/>
-      <c r="E129" s="7"/>
-    </row>
-    <row r="130" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B130" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="131" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B131" t="s">
+      <c r="E129" s="4"/>
+    </row>
+    <row r="130" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B130" s="4" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="132" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B132" t="s">
+      <c r="C130" s="4"/>
+      <c r="D130" s="5"/>
+      <c r="E130" s="4"/>
+    </row>
+    <row r="131" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B131" s="4" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="133" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B133" t="s">
+      <c r="C131" s="4"/>
+      <c r="D131" s="5"/>
+      <c r="E131" s="4"/>
+    </row>
+    <row r="132" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B132" s="4" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="134" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B134" t="s">
+      <c r="C132" s="4"/>
+      <c r="D132" s="5"/>
+      <c r="E132" s="4"/>
+    </row>
+    <row r="133" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B133" s="4" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="135" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B135" t="s">
+      <c r="C133" s="4"/>
+      <c r="D133" s="5"/>
+      <c r="E133" s="4"/>
+    </row>
+    <row r="134" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B134" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="C134" s="4"/>
+      <c r="D134" s="5"/>
+      <c r="E134" s="4"/>
+    </row>
+    <row r="135" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B135" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C135" s="4"/>
+      <c r="D135" s="5"/>
+      <c r="E135" s="4"/>
+    </row>
+    <row r="136" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B136" s="4" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="136" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B136" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="137" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B137" t="s">
+      <c r="C136" s="4"/>
+      <c r="D136" s="5"/>
+      <c r="E136" s="4"/>
+    </row>
+    <row r="137" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B137" s="4" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="138" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B138" t="s">
+      <c r="C137" s="4"/>
+      <c r="D137" s="5"/>
+      <c r="E137" s="4"/>
+    </row>
+    <row r="138" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B138" s="4" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="139" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B139" t="s">
+      <c r="C138" s="4"/>
+      <c r="D138" s="5"/>
+      <c r="E138" s="4"/>
+    </row>
+    <row r="139" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B139" s="4" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="140" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B140" t="s">
+      <c r="C139" s="4"/>
+      <c r="D139" s="5"/>
+      <c r="E139" s="4"/>
+    </row>
+    <row r="140" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B140" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="C140" s="4"/>
+      <c r="D140" s="5"/>
+      <c r="E140" s="4"/>
+    </row>
+    <row r="141" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B141" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C141" s="4"/>
+      <c r="D141" s="5"/>
+      <c r="E141" s="4"/>
+    </row>
+    <row r="142" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B142" s="4" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="141" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B141" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="142" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B142" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="143" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B143" t="s">
+      <c r="C142" s="4"/>
+      <c r="D142" s="5"/>
+      <c r="E142" s="4"/>
+    </row>
+    <row r="143" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B143" s="4" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="144" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B144" t="s">
+      <c r="C143" s="4"/>
+      <c r="D143" s="5"/>
+      <c r="E143" s="4"/>
+    </row>
+    <row r="144" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B144" s="4" t="s">
         <v>189</v>
       </c>
-    </row>
-    <row r="145" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B145" t="s">
+      <c r="C144" s="4"/>
+      <c r="D144" s="5"/>
+      <c r="E144" s="4"/>
+    </row>
+    <row r="145" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B145" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="C145" s="4"/>
+      <c r="D145" s="5"/>
+      <c r="E145" s="4"/>
+    </row>
+    <row r="146" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B146" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C146" s="4"/>
+      <c r="D146" s="5"/>
+      <c r="E146" s="4"/>
+    </row>
+    <row r="147" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B147" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C147" s="4"/>
+      <c r="D147" s="5"/>
+      <c r="E147" s="4"/>
+    </row>
+    <row r="148" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B148" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C148" s="4"/>
+      <c r="D148" s="5"/>
+      <c r="E148" s="4"/>
+    </row>
+    <row r="149" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B149" s="4" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="146" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B146" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="147" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B147" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="148" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B148" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="149" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B149" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="150" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B150" t="s">
+      <c r="C149" s="4"/>
+      <c r="D149" s="5"/>
+      <c r="E149" s="4"/>
+    </row>
+    <row r="150" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B150" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C150" s="4"/>
+      <c r="D150" s="5"/>
+      <c r="E150" s="4"/>
+    </row>
+    <row r="151" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B151" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C151" s="4"/>
+      <c r="D151" s="5"/>
+      <c r="E151" s="4"/>
+    </row>
+    <row r="152" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B152" s="4" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="151" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B151" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="152" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B152" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="153" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B153" t="s">
+      <c r="C152" s="4"/>
+      <c r="D152" s="5"/>
+      <c r="E152" s="4"/>
+    </row>
+    <row r="153" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B153" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="C153" s="4"/>
+      <c r="D153" s="5"/>
+      <c r="E153" s="4"/>
+    </row>
+    <row r="154" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B154" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C154" s="4"/>
+      <c r="D154" s="5"/>
+      <c r="E154" s="4"/>
+    </row>
+    <row r="155" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B155" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C155" s="4"/>
+      <c r="D155" s="5"/>
+      <c r="E155" s="4"/>
+    </row>
+    <row r="156" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B156" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C156" s="4"/>
+      <c r="D156" s="5"/>
+      <c r="E156" s="4"/>
+    </row>
+    <row r="157" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B157" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C157" s="4"/>
+      <c r="D157" s="5"/>
+      <c r="E157" s="4"/>
+    </row>
+    <row r="158" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B158" s="4" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="154" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B154" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="155" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B155" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="156" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B156" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="157" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B157" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="158" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B158" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="159" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B159" t="s">
+      <c r="C158" s="4"/>
+      <c r="D158" s="5"/>
+      <c r="E158" s="4"/>
+    </row>
+    <row r="159" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B159" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C159" s="4"/>
+      <c r="D159" s="5"/>
+      <c r="E159" s="4"/>
+    </row>
+    <row r="160" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B160" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C160" s="4"/>
+      <c r="D160" s="5"/>
+      <c r="E160" s="4"/>
+    </row>
+    <row r="161" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B161" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="C161" s="4"/>
+      <c r="D161" s="5"/>
+      <c r="E161" s="4"/>
+    </row>
+    <row r="162" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B162" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="C162" s="4"/>
+      <c r="D162" s="5"/>
+      <c r="E162" s="4"/>
+    </row>
+    <row r="163" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B163" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="C163" s="4"/>
+      <c r="D163" s="5"/>
+      <c r="E163" s="4"/>
+    </row>
+    <row r="164" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B164" s="4" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="160" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B160" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="161" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B161" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="162" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B162" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="163" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B163" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="164" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B164" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="165" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B165" t="s">
+      <c r="C164" s="4"/>
+      <c r="D164" s="5"/>
+      <c r="E164" s="4"/>
+    </row>
+    <row r="165" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B165" s="4" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="166" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B166" t="s">
+      <c r="C165" s="4"/>
+      <c r="D165" s="5"/>
+      <c r="E165" s="4"/>
+    </row>
+    <row r="166" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B166" s="4" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="167" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B167" t="s">
+      <c r="C166" s="4"/>
+      <c r="D166" s="5"/>
+      <c r="E166" s="4"/>
+    </row>
+    <row r="167" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B167" s="4" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="168" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B168" t="s">
+      <c r="C167" s="4"/>
+      <c r="D167" s="5"/>
+      <c r="E167" s="4"/>
+    </row>
+    <row r="168" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B168" s="4" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="169" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B169" t="s">
+      <c r="C168" s="4"/>
+      <c r="D168" s="5"/>
+      <c r="E168" s="4"/>
+    </row>
+    <row r="169" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B169" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="C169" s="4"/>
+      <c r="D169" s="5"/>
+      <c r="E169" s="4"/>
+    </row>
+    <row r="170" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B170" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="C170" s="4"/>
+      <c r="D170" s="5"/>
+      <c r="E170" s="4"/>
+    </row>
+    <row r="171" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B171" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C171" s="4"/>
+      <c r="D171" s="5"/>
+      <c r="E171" s="4"/>
+    </row>
+    <row r="172" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B172" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="C172" s="4"/>
+      <c r="D172" s="5"/>
+      <c r="E172" s="4"/>
+    </row>
+    <row r="173" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B173" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C173" s="4"/>
+      <c r="D173" s="5"/>
+      <c r="E173" s="4"/>
+    </row>
+    <row r="174" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B174" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="C174" s="4"/>
+      <c r="D174" s="5"/>
+      <c r="E174" s="4"/>
+    </row>
+    <row r="175" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B175" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C175" s="4"/>
+      <c r="D175" s="5"/>
+      <c r="E175" s="4"/>
+    </row>
+    <row r="176" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B176" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="C176" s="4"/>
+      <c r="D176" s="5"/>
+      <c r="E176" s="4"/>
+    </row>
+    <row r="177" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B177" s="4" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="170" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B170" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="171" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B171" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="172" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B172" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="173" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B173" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="174" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B174" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="175" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B175" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="176" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B176" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="177" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B177" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="178" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B178" t="s">
+      <c r="C177" s="4"/>
+      <c r="D177" s="5"/>
+      <c r="E177" s="4"/>
+    </row>
+    <row r="178" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B178" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C178" s="4"/>
+      <c r="D178" s="5"/>
+      <c r="E178" s="4"/>
+    </row>
+    <row r="179" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B179" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="C179" s="4"/>
+      <c r="D179" s="5"/>
+      <c r="E179" s="4"/>
+    </row>
+    <row r="180" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B180" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C180" s="4"/>
+      <c r="D180" s="5"/>
+      <c r="E180" s="4"/>
+    </row>
+    <row r="181" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B181" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="C181" s="4"/>
+      <c r="D181" s="5"/>
+      <c r="E181" s="4"/>
+    </row>
+    <row r="182" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B182" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C182" s="4"/>
+      <c r="D182" s="5"/>
+      <c r="E182" s="4"/>
+    </row>
+    <row r="183" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B183" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C183" s="4"/>
+      <c r="D183" s="5"/>
+      <c r="E183" s="4"/>
+    </row>
+    <row r="184" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B184" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="C184" s="4"/>
+      <c r="D184" s="5"/>
+      <c r="E184" s="4"/>
+    </row>
+    <row r="185" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B185" s="4" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="179" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B179" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="180" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B180" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="181" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B181" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="182" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B182" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="183" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B183" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="184" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B184" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="185" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B185" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="186" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B186" t="s">
+      <c r="C185" s="4"/>
+      <c r="D185" s="5"/>
+      <c r="E185" s="4"/>
+    </row>
+    <row r="186" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B186" s="4" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="187" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B187" t="s">
+      <c r="C186" s="4"/>
+      <c r="D186" s="5"/>
+      <c r="E186" s="4"/>
+    </row>
+    <row r="187" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B187" s="4" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="188" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B188" t="s">
+      <c r="C187" s="4"/>
+      <c r="D187" s="5"/>
+      <c r="E187" s="4"/>
+    </row>
+    <row r="188" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B188" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="C188" s="4"/>
+      <c r="D188" s="5"/>
+      <c r="E188" s="4"/>
+    </row>
+    <row r="189" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B189" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C189" s="4"/>
+      <c r="D189" s="5"/>
+      <c r="E189" s="4"/>
+    </row>
+    <row r="190" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B190" s="4" t="s">
         <v>202</v>
       </c>
-    </row>
-    <row r="189" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B189" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="190" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B190" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="191" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B191" t="s">
+      <c r="C190" s="4"/>
+      <c r="D190" s="5"/>
+      <c r="E190" s="4"/>
+    </row>
+    <row r="191" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B191" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="C191" s="4"/>
+      <c r="D191" s="5"/>
+      <c r="E191" s="4"/>
+    </row>
+    <row r="192" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B192" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="C192" s="4"/>
+      <c r="D192" s="5"/>
+      <c r="E192" s="4"/>
+    </row>
+    <row r="193" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B193" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="C193" s="4"/>
+      <c r="D193" s="5"/>
+      <c r="E193" s="4"/>
+    </row>
+    <row r="194" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B194" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="C194" s="4"/>
+      <c r="D194" s="5"/>
+      <c r="E194" s="4"/>
+    </row>
+    <row r="195" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B195" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="C195" s="4"/>
+      <c r="D195" s="5"/>
+      <c r="E195" s="4"/>
+    </row>
+    <row r="196" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B196" s="4" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="192" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B192" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="193" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B193" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="194" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B194" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="195" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B195" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="196" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B196" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="197" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B197" t="s">
+      <c r="C196" s="4"/>
+      <c r="D196" s="5"/>
+      <c r="E196" s="4"/>
+    </row>
+    <row r="197" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B197" s="4" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="198" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B198" t="s">
+      <c r="C197" s="4"/>
+      <c r="D197" s="5"/>
+      <c r="E197" s="4"/>
+    </row>
+    <row r="198" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B198" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="C198" s="4"/>
+      <c r="D198" s="5"/>
+      <c r="E198" s="4"/>
+    </row>
+    <row r="199" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B199" s="4" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="199" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B199" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="200" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B200" t="s">
+      <c r="C199" s="4"/>
+      <c r="D199" s="5"/>
+      <c r="E199" s="4"/>
+    </row>
+    <row r="200" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B200" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="C200" s="4"/>
+      <c r="D200" s="5"/>
+      <c r="E200" s="4"/>
+    </row>
+    <row r="201" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B201" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C201" s="4"/>
+      <c r="D201" s="5"/>
+      <c r="E201" s="4"/>
+    </row>
+    <row r="202" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B202" s="4" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="201" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B201" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="202" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B202" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="203" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B203" t="s">
+      <c r="C202" s="4"/>
+      <c r="D202" s="5"/>
+      <c r="E202" s="4"/>
+    </row>
+    <row r="203" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B203" s="4" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="204" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B204" t="s">
-        <v>208</v>
-      </c>
+      <c r="C203" s="4"/>
+      <c r="D203" s="5"/>
+      <c r="E203" s="4"/>
+    </row>
+    <row r="204" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D204" s="1"/>
+    </row>
+    <row r="205" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D205" s="1"/>
+    </row>
+    <row r="206" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D206" s="1"/>
+    </row>
+    <row r="207" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D207" s="1"/>
+    </row>
+    <row r="208" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D208" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup scale="32" fitToWidth="0" fitToHeight="0" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Se hizo cambios en los archivos JSP se implemento el metodo del constructor de consultas y en ese archivo se agrego ? en las variables.
</commit_message>
<xml_diff>
--- a/Control.xlsx
+++ b/Control.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\10.106.12.32\compartir\openlayers2_nvo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{526BABFF-BB27-4798-BE81-221A2BF88BC2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E3302B5-894B-42B6-AE80-012ACC8CAA4B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="13905" xr2:uid="{119285BF-BAF3-43BB-BF3D-96AE8CA3F258}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15345" windowHeight="4380" xr2:uid="{119285BF-BAF3-43BB-BF3D-96AE8CA3F258}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="210">
   <si>
     <t>agregacgo.jsp</t>
   </si>
@@ -652,6 +652,9 @@
   </si>
   <si>
     <t>Ricardo</t>
+  </si>
+  <si>
+    <t>No tiene consultas</t>
   </si>
 </sst>
 </file>
@@ -736,7 +739,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -758,6 +761,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Bueno" xfId="1" builtinId="26"/>
@@ -1108,7 +1113,7 @@
       <c r="B2" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="C2" s="2"/>
+      <c r="C2" s="10"/>
       <c r="D2" s="5" t="s">
         <v>208</v>
       </c>
@@ -1120,40 +1125,50 @@
       <c r="B3" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="C3" s="4"/>
+      <c r="C3" s="9"/>
       <c r="D3" s="5"/>
-      <c r="E3" s="7"/>
+      <c r="E3" s="7" t="s">
+        <v>209</v>
+      </c>
     </row>
     <row r="4" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="4"/>
-      <c r="D4" s="5"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="5" t="s">
+        <v>208</v>
+      </c>
       <c r="E4" s="7"/>
     </row>
     <row r="5" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="C5" s="4"/>
+      <c r="C5" s="10"/>
       <c r="D5" s="5"/>
-      <c r="E5" s="7"/>
+      <c r="E5" s="7" t="s">
+        <v>209</v>
+      </c>
     </row>
     <row r="6" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="C6" s="4"/>
+      <c r="C6" s="9"/>
       <c r="D6" s="5"/>
-      <c r="E6" s="7"/>
+      <c r="E6" s="7" t="s">
+        <v>209</v>
+      </c>
     </row>
     <row r="7" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="5"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="5" t="s">
+        <v>208</v>
+      </c>
       <c r="E7" s="7"/>
     </row>
     <row r="8" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Se modifico el archivo jsp de acuerdo al constructor de consultas
</commit_message>
<xml_diff>
--- a/Control.xlsx
+++ b/Control.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\10.106.12.32\compartir\openlayers2_nvo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E3302B5-894B-42B6-AE80-012ACC8CAA4B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1971EBCA-091D-4D73-9C86-501008A2372E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="15345" windowHeight="4380" xr2:uid="{119285BF-BAF3-43BB-BF3D-96AE8CA3F258}"/>
   </bookViews>
@@ -1175,7 +1175,7 @@
       <c r="B8" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C8" s="4"/>
+      <c r="C8" s="10"/>
       <c r="D8" s="5"/>
       <c r="E8" s="7"/>
     </row>

</xml_diff>

<commit_message>
Se corrigieron los primeros archivos cerrando la conexion, en los demas archivos se agrego la consulta al constructor y en el jsp se agrego el metodo de la consulta.
</commit_message>
<xml_diff>
--- a/Control.xlsx
+++ b/Control.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\10.106.12.32\compartir\openlayers2_nvo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1971EBCA-091D-4D73-9C86-501008A2372E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52EE8346-4789-4EC8-9DF3-D4FCA8A9BB78}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15345" windowHeight="4380" xr2:uid="{119285BF-BAF3-43BB-BF3D-96AE8CA3F258}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="13905" xr2:uid="{119285BF-BAF3-43BB-BF3D-96AE8CA3F258}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="211">
   <si>
     <t>agregacgo.jsp</t>
   </si>
@@ -655,6 +655,9 @@
   </si>
   <si>
     <t>No tiene consultas</t>
+  </si>
+  <si>
+    <t>No ejecuta consulta</t>
   </si>
 </sst>
 </file>
@@ -739,7 +742,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -763,6 +766,7 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="2" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Bueno" xfId="1" builtinId="26"/>
@@ -1176,87 +1180,109 @@
         <v>2</v>
       </c>
       <c r="C8" s="10"/>
-      <c r="D8" s="5"/>
+      <c r="D8" s="5" t="s">
+        <v>208</v>
+      </c>
       <c r="E8" s="7"/>
     </row>
     <row r="9" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C9" s="4"/>
-      <c r="D9" s="5"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="5" t="s">
+        <v>208</v>
+      </c>
       <c r="E9" s="7"/>
     </row>
     <row r="10" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C10" s="4"/>
-      <c r="D10" s="5"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="5" t="s">
+        <v>208</v>
+      </c>
       <c r="E10" s="7"/>
     </row>
     <row r="11" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C11" s="4"/>
-      <c r="D11" s="5"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="5" t="s">
+        <v>208</v>
+      </c>
       <c r="E11" s="7"/>
     </row>
     <row r="12" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="4"/>
-      <c r="D12" s="5"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="5" t="s">
+        <v>208</v>
+      </c>
       <c r="E12" s="7"/>
     </row>
     <row r="13" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="4"/>
+      <c r="C13" s="10"/>
       <c r="D13" s="5"/>
-      <c r="E13" s="7"/>
+      <c r="E13" s="7" t="s">
+        <v>210</v>
+      </c>
     </row>
     <row r="14" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C14" s="4"/>
-      <c r="D14" s="5"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="5" t="s">
+        <v>208</v>
+      </c>
       <c r="E14" s="7"/>
     </row>
     <row r="15" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C15" s="4"/>
-      <c r="D15" s="5"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="5" t="s">
+        <v>208</v>
+      </c>
       <c r="E15" s="7"/>
     </row>
     <row r="16" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C16" s="4"/>
-      <c r="D16" s="5"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="5" t="s">
+        <v>208</v>
+      </c>
       <c r="E16" s="7"/>
     </row>
     <row r="17" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="C17" s="4"/>
+      <c r="C17" s="10"/>
       <c r="D17" s="5"/>
-      <c r="E17" s="7"/>
+      <c r="E17" s="7" t="s">
+        <v>210</v>
+      </c>
     </row>
     <row r="18" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C18" s="4"/>
-      <c r="D18" s="5"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="5" t="s">
+        <v>208</v>
+      </c>
       <c r="E18" s="7"/>
     </row>
     <row r="19" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Se regenero el proyecto debido a errores para encontrar las clases
</commit_message>
<xml_diff>
--- a/Control.xlsx
+++ b/Control.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\10.106.12.32\compartir\openlayers2_nvo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52EE8346-4789-4EC8-9DF3-D4FCA8A9BB78}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3722E00-718B-45CB-9DED-7A25E1FCEDA5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="13905" xr2:uid="{119285BF-BAF3-43BB-BF3D-96AE8CA3F258}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15345" windowHeight="4380" xr2:uid="{119285BF-BAF3-43BB-BF3D-96AE8CA3F258}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -1289,7 +1289,7 @@
       <c r="B19" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C19" s="4"/>
+      <c r="C19" s="10"/>
       <c r="D19" s="5"/>
       <c r="E19" s="7"/>
     </row>
@@ -1297,7 +1297,7 @@
       <c r="B20" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C20" s="4"/>
+      <c r="C20" s="10"/>
       <c r="D20" s="5"/>
       <c r="E20" s="7"/>
     </row>
@@ -1305,7 +1305,7 @@
       <c r="B21" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C21" s="4"/>
+      <c r="C21" s="10"/>
       <c r="D21" s="5"/>
       <c r="E21" s="7"/>
     </row>
@@ -1313,7 +1313,7 @@
       <c r="B22" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="C22" s="4"/>
+      <c r="C22" s="10"/>
       <c r="D22" s="5"/>
       <c r="E22" s="7"/>
     </row>

</xml_diff>

<commit_message>
Indice ya con clases java
</commit_message>
<xml_diff>
--- a/Control.xlsx
+++ b/Control.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\10.106.12.32\compartir\openlayers2_nvo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\compartir\openlayers2_nvo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3722E00-718B-45CB-9DED-7A25E1FCEDA5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F96190D-6215-480E-B7E9-15B9F1A20041}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15345" windowHeight="4380" xr2:uid="{119285BF-BAF3-43BB-BF3D-96AE8CA3F258}"/>
+    <workbookView xWindow="1125" yWindow="1245" windowWidth="25860" windowHeight="11295" xr2:uid="{119285BF-BAF3-43BB-BF3D-96AE8CA3F258}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="213">
   <si>
     <t>agregacgo.jsp</t>
   </si>
@@ -658,13 +658,19 @@
   </si>
   <si>
     <t>No ejecuta consulta</t>
+  </si>
+  <si>
+    <t>Arturo</t>
+  </si>
+  <si>
+    <t>Indice ya quedo usando conn. Pool</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -689,6 +695,13 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -742,7 +755,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -767,6 +780,9 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Bueno" xfId="1" builtinId="26"/>
@@ -787,9 +803,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -827,7 +843,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -933,7 +949,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1075,7 +1091,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1617,9 +1633,13 @@
       <c r="B60" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C60" s="4"/>
-      <c r="D60" s="5"/>
-      <c r="E60" s="7"/>
+      <c r="C60" s="10"/>
+      <c r="D60" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="E60" s="12" t="s">
+        <v>212</v>
+      </c>
     </row>
     <row r="61" spans="2:5" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B61" s="4" t="s">

</xml_diff>

<commit_message>
Se movieron las consultas al constructor de consultas de los archivos jsp
</commit_message>
<xml_diff>
--- a/Control.xlsx
+++ b/Control.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\compartir\openlayers2_nvo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\10.106.12.32\compartir\openlayers2_nvo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FEE646A-C9E0-4FDA-A26B-CB74F00B7917}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{866FF221-E1A1-475E-887A-A3F8D7BEFA47}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1125" yWindow="1245" windowWidth="25860" windowHeight="11295" xr2:uid="{119285BF-BAF3-43BB-BF3D-96AE8CA3F258}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="13905" xr2:uid="{119285BF-BAF3-43BB-BF3D-96AE8CA3F258}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja2" sheetId="2" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="220">
   <si>
     <t>agregacgo.jsp</t>
   </si>
@@ -824,9 +824,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -864,7 +864,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -970,7 +970,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1112,7 +1112,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1308,7 +1308,9 @@
         <v>12</v>
       </c>
       <c r="D15" s="10"/>
-      <c r="E15" s="5"/>
+      <c r="E15" s="5" t="s">
+        <v>208</v>
+      </c>
       <c r="F15" s="7"/>
       <c r="G15" s="5">
         <v>1</v>
@@ -1319,7 +1321,9 @@
         <v>13</v>
       </c>
       <c r="D16" s="10"/>
-      <c r="E16" s="5"/>
+      <c r="E16" s="5" t="s">
+        <v>208</v>
+      </c>
       <c r="F16" s="7"/>
       <c r="G16" s="5">
         <v>1</v>
@@ -1330,7 +1334,9 @@
         <v>14</v>
       </c>
       <c r="D17" s="10"/>
-      <c r="E17" s="5"/>
+      <c r="E17" s="5" t="s">
+        <v>208</v>
+      </c>
       <c r="F17" s="7"/>
       <c r="G17" s="5">
         <v>1</v>
@@ -1341,7 +1347,9 @@
         <v>136</v>
       </c>
       <c r="D18" s="10"/>
-      <c r="E18" s="5"/>
+      <c r="E18" s="5" t="s">
+        <v>208</v>
+      </c>
       <c r="F18" s="7"/>
       <c r="G18" s="5">
         <v>1</v>
@@ -1352,7 +1360,9 @@
         <v>15</v>
       </c>
       <c r="D19" s="10"/>
-      <c r="E19" s="5"/>
+      <c r="E19" s="5" t="s">
+        <v>208</v>
+      </c>
       <c r="F19" s="7"/>
       <c r="G19" s="5">
         <v>1</v>
@@ -1363,7 +1373,9 @@
         <v>16</v>
       </c>
       <c r="D20" s="10"/>
-      <c r="E20" s="5"/>
+      <c r="E20" s="5" t="s">
+        <v>208</v>
+      </c>
       <c r="F20" s="7"/>
       <c r="G20" s="5">
         <v>1</v>
@@ -1374,7 +1386,9 @@
         <v>17</v>
       </c>
       <c r="D21" s="10"/>
-      <c r="E21" s="5"/>
+      <c r="E21" s="5" t="s">
+        <v>208</v>
+      </c>
       <c r="F21" s="7"/>
       <c r="G21" s="5">
         <v>1</v>
@@ -1385,7 +1399,9 @@
         <v>137</v>
       </c>
       <c r="D22" s="10"/>
-      <c r="E22" s="4"/>
+      <c r="E22" s="5" t="s">
+        <v>208</v>
+      </c>
       <c r="F22" s="4"/>
       <c r="G22" s="5">
         <v>1</v>
@@ -1396,7 +1412,9 @@
         <v>138</v>
       </c>
       <c r="D23" s="10"/>
-      <c r="E23" s="4"/>
+      <c r="E23" s="5" t="s">
+        <v>208</v>
+      </c>
       <c r="F23" s="4"/>
       <c r="G23" s="5">
         <v>1</v>
@@ -1407,7 +1425,9 @@
         <v>18</v>
       </c>
       <c r="D24" s="10"/>
-      <c r="E24" s="4"/>
+      <c r="E24" s="5" t="s">
+        <v>208</v>
+      </c>
       <c r="F24" s="4"/>
       <c r="G24" s="5">
         <v>1</v>
@@ -1418,7 +1438,9 @@
         <v>19</v>
       </c>
       <c r="D25" s="10"/>
-      <c r="E25" s="4"/>
+      <c r="E25" s="5" t="s">
+        <v>208</v>
+      </c>
       <c r="F25" s="4"/>
       <c r="G25" s="5">
         <v>1</v>
@@ -1428,46 +1450,66 @@
       <c r="C26" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="D26" s="4"/>
-      <c r="E26" s="4"/>
+      <c r="D26" s="10"/>
+      <c r="E26" s="5" t="s">
+        <v>208</v>
+      </c>
       <c r="F26" s="4"/>
-      <c r="G26" s="4"/>
+      <c r="G26" s="5">
+        <v>2</v>
+      </c>
     </row>
     <row r="27" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C27" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D27" s="4"/>
-      <c r="E27" s="4"/>
+      <c r="D27" s="10"/>
+      <c r="E27" s="5" t="s">
+        <v>208</v>
+      </c>
       <c r="F27" s="4"/>
-      <c r="G27" s="4"/>
+      <c r="G27" s="5">
+        <v>2</v>
+      </c>
     </row>
     <row r="28" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C28" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D28" s="4"/>
-      <c r="E28" s="4"/>
+      <c r="D28" s="10"/>
+      <c r="E28" s="5" t="s">
+        <v>208</v>
+      </c>
       <c r="F28" s="4"/>
-      <c r="G28" s="4"/>
+      <c r="G28" s="5">
+        <v>2</v>
+      </c>
     </row>
     <row r="29" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C29" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D29" s="4"/>
-      <c r="E29" s="4"/>
+      <c r="D29" s="10"/>
+      <c r="E29" s="5" t="s">
+        <v>208</v>
+      </c>
       <c r="F29" s="4"/>
-      <c r="G29" s="4"/>
+      <c r="G29" s="5">
+        <v>2</v>
+      </c>
     </row>
     <row r="30" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C30" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D30" s="4"/>
-      <c r="E30" s="4"/>
+      <c r="D30" s="10"/>
+      <c r="E30" s="5" t="s">
+        <v>208</v>
+      </c>
       <c r="F30" s="4"/>
-      <c r="G30" s="4"/>
+      <c r="G30" s="5">
+        <v>2</v>
+      </c>
     </row>
     <row r="31" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C31" s="4" t="s">
@@ -1476,7 +1518,7 @@
       <c r="D31" s="4"/>
       <c r="E31" s="4"/>
       <c r="F31" s="4"/>
-      <c r="G31" s="4"/>
+      <c r="G31" s="5"/>
     </row>
     <row r="32" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C32" s="4" t="s">
@@ -1485,7 +1527,7 @@
       <c r="D32" s="4"/>
       <c r="E32" s="4"/>
       <c r="F32" s="4"/>
-      <c r="G32" s="4"/>
+      <c r="G32" s="5"/>
     </row>
     <row r="33" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C33" s="4" t="s">
@@ -1494,7 +1536,7 @@
       <c r="D33" s="4"/>
       <c r="E33" s="4"/>
       <c r="F33" s="4"/>
-      <c r="G33" s="4"/>
+      <c r="G33" s="5"/>
     </row>
     <row r="34" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C34" s="4" t="s">
@@ -1503,7 +1545,7 @@
       <c r="D34" s="4"/>
       <c r="E34" s="4"/>
       <c r="F34" s="4"/>
-      <c r="G34" s="4"/>
+      <c r="G34" s="5"/>
     </row>
     <row r="35" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C35" s="4" t="s">
@@ -1512,7 +1554,7 @@
       <c r="D35" s="4"/>
       <c r="E35" s="4"/>
       <c r="F35" s="4"/>
-      <c r="G35" s="4"/>
+      <c r="G35" s="5"/>
     </row>
     <row r="36" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C36" s="4" t="s">
@@ -1521,7 +1563,7 @@
       <c r="D36" s="4"/>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
-      <c r="G36" s="4"/>
+      <c r="G36" s="5"/>
     </row>
     <row r="37" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C37" s="4" t="s">
@@ -1530,7 +1572,7 @@
       <c r="D37" s="4"/>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
-      <c r="G37" s="4"/>
+      <c r="G37" s="5"/>
     </row>
     <row r="38" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C38" s="4" t="s">
@@ -1543,7 +1585,7 @@
       <c r="F38" s="12" t="s">
         <v>212</v>
       </c>
-      <c r="G38" s="4"/>
+      <c r="G38" s="5"/>
     </row>
     <row r="39" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C39" s="4" t="s">
@@ -1552,7 +1594,7 @@
       <c r="D39" s="4"/>
       <c r="E39" s="4"/>
       <c r="F39" s="4"/>
-      <c r="G39" s="4"/>
+      <c r="G39" s="5"/>
     </row>
     <row r="40" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C40" s="4" t="s">
@@ -1561,7 +1603,7 @@
       <c r="D40" s="4"/>
       <c r="E40" s="4"/>
       <c r="F40" s="4"/>
-      <c r="G40" s="4"/>
+      <c r="G40" s="5"/>
     </row>
     <row r="41" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C41" s="4" t="s">
@@ -1570,7 +1612,7 @@
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
       <c r="F41" s="4"/>
-      <c r="G41" s="4"/>
+      <c r="G41" s="5"/>
     </row>
     <row r="42" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C42" s="4" t="s">
@@ -1579,7 +1621,7 @@
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>
       <c r="F42" s="4"/>
-      <c r="G42" s="4"/>
+      <c r="G42" s="5"/>
     </row>
     <row r="43" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C43" s="4" t="s">
@@ -1588,7 +1630,7 @@
       <c r="D43" s="4"/>
       <c r="E43" s="4"/>
       <c r="F43" s="4"/>
-      <c r="G43" s="4"/>
+      <c r="G43" s="5"/>
     </row>
     <row r="44" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C44" s="4" t="s">
@@ -1597,7 +1639,7 @@
       <c r="D44" s="4"/>
       <c r="E44" s="4"/>
       <c r="F44" s="4"/>
-      <c r="G44" s="4"/>
+      <c r="G44" s="5"/>
     </row>
     <row r="45" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C45" s="4" t="s">
@@ -1606,7 +1648,7 @@
       <c r="D45" s="4"/>
       <c r="E45" s="4"/>
       <c r="F45" s="4"/>
-      <c r="G45" s="4"/>
+      <c r="G45" s="5"/>
     </row>
     <row r="46" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C46" s="4" t="s">
@@ -1615,7 +1657,7 @@
       <c r="D46" s="4"/>
       <c r="E46" s="4"/>
       <c r="F46" s="4"/>
-      <c r="G46" s="4"/>
+      <c r="G46" s="5"/>
     </row>
     <row r="47" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C47" s="4" t="s">
@@ -1624,7 +1666,7 @@
       <c r="D47" s="4"/>
       <c r="E47" s="4"/>
       <c r="F47" s="4"/>
-      <c r="G47" s="4"/>
+      <c r="G47" s="5"/>
     </row>
     <row r="48" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C48" s="4" t="s">
@@ -1633,7 +1675,7 @@
       <c r="D48" s="4"/>
       <c r="E48" s="4"/>
       <c r="F48" s="4"/>
-      <c r="G48" s="4"/>
+      <c r="G48" s="5"/>
     </row>
     <row r="49" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C49" s="4" t="s">
@@ -1642,7 +1684,7 @@
       <c r="D49" s="4"/>
       <c r="E49" s="4"/>
       <c r="F49" s="4"/>
-      <c r="G49" s="4"/>
+      <c r="G49" s="5"/>
     </row>
     <row r="50" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C50" s="4" t="s">
@@ -1651,7 +1693,7 @@
       <c r="D50" s="4"/>
       <c r="E50" s="4"/>
       <c r="F50" s="4"/>
-      <c r="G50" s="4"/>
+      <c r="G50" s="5"/>
     </row>
     <row r="51" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C51" s="4" t="s">
@@ -1660,7 +1702,7 @@
       <c r="D51" s="4"/>
       <c r="E51" s="4"/>
       <c r="F51" s="4"/>
-      <c r="G51" s="4"/>
+      <c r="G51" s="5"/>
     </row>
     <row r="52" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C52" s="4" t="s">
@@ -1669,7 +1711,7 @@
       <c r="D52" s="4"/>
       <c r="E52" s="4"/>
       <c r="F52" s="4"/>
-      <c r="G52" s="4"/>
+      <c r="G52" s="5"/>
     </row>
     <row r="53" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C53" s="4" t="s">
@@ -1678,7 +1720,7 @@
       <c r="D53" s="4"/>
       <c r="E53" s="4"/>
       <c r="F53" s="4"/>
-      <c r="G53" s="4"/>
+      <c r="G53" s="5"/>
     </row>
     <row r="54" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C54" s="4" t="s">
@@ -1687,7 +1729,7 @@
       <c r="D54" s="4"/>
       <c r="E54" s="4"/>
       <c r="F54" s="4"/>
-      <c r="G54" s="4"/>
+      <c r="G54" s="5"/>
     </row>
     <row r="55" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C55" s="4" t="s">
@@ -1696,7 +1738,7 @@
       <c r="D55" s="4"/>
       <c r="E55" s="4"/>
       <c r="F55" s="4"/>
-      <c r="G55" s="4"/>
+      <c r="G55" s="5"/>
     </row>
     <row r="56" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C56" s="4" t="s">
@@ -1705,7 +1747,7 @@
       <c r="D56" s="4"/>
       <c r="E56" s="4"/>
       <c r="F56" s="4"/>
-      <c r="G56" s="4"/>
+      <c r="G56" s="5"/>
     </row>
     <row r="57" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C57" s="4" t="s">
@@ -1714,7 +1756,7 @@
       <c r="D57" s="4"/>
       <c r="E57" s="4"/>
       <c r="F57" s="4"/>
-      <c r="G57" s="4"/>
+      <c r="G57" s="5"/>
     </row>
     <row r="58" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C58" s="4" t="s">
@@ -1723,7 +1765,7 @@
       <c r="D58" s="4"/>
       <c r="E58" s="4"/>
       <c r="F58" s="4"/>
-      <c r="G58" s="4"/>
+      <c r="G58" s="5"/>
     </row>
     <row r="59" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C59" s="4" t="s">
@@ -1732,7 +1774,7 @@
       <c r="D59" s="4"/>
       <c r="E59" s="4"/>
       <c r="F59" s="4"/>
-      <c r="G59" s="4"/>
+      <c r="G59" s="5"/>
     </row>
     <row r="60" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C60" s="4" t="s">
@@ -1741,7 +1783,7 @@
       <c r="D60" s="4"/>
       <c r="E60" s="4"/>
       <c r="F60" s="4"/>
-      <c r="G60" s="4"/>
+      <c r="G60" s="5"/>
     </row>
     <row r="61" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C61" s="4" t="s">
@@ -1750,7 +1792,7 @@
       <c r="D61" s="4"/>
       <c r="E61" s="4"/>
       <c r="F61" s="4"/>
-      <c r="G61" s="4"/>
+      <c r="G61" s="5"/>
     </row>
     <row r="62" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C62" s="4" t="s">
@@ -1759,7 +1801,7 @@
       <c r="D62" s="4"/>
       <c r="E62" s="4"/>
       <c r="F62" s="4"/>
-      <c r="G62" s="4"/>
+      <c r="G62" s="5"/>
     </row>
     <row r="63" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C63" s="4" t="s">
@@ -1768,7 +1810,7 @@
       <c r="D63" s="4"/>
       <c r="E63" s="4"/>
       <c r="F63" s="4"/>
-      <c r="G63" s="4"/>
+      <c r="G63" s="5"/>
     </row>
     <row r="64" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C64" s="4" t="s">
@@ -1777,7 +1819,7 @@
       <c r="D64" s="4"/>
       <c r="E64" s="4"/>
       <c r="F64" s="4"/>
-      <c r="G64" s="4"/>
+      <c r="G64" s="5"/>
     </row>
     <row r="65" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C65" s="4" t="s">
@@ -1786,7 +1828,7 @@
       <c r="D65" s="4"/>
       <c r="E65" s="4"/>
       <c r="F65" s="4"/>
-      <c r="G65" s="4"/>
+      <c r="G65" s="5"/>
     </row>
     <row r="66" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C66" s="4" t="s">
@@ -1795,7 +1837,7 @@
       <c r="D66" s="4"/>
       <c r="E66" s="4"/>
       <c r="F66" s="4"/>
-      <c r="G66" s="4"/>
+      <c r="G66" s="5"/>
     </row>
     <row r="67" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C67" s="4" t="s">
@@ -1804,7 +1846,7 @@
       <c r="D67" s="4"/>
       <c r="E67" s="4"/>
       <c r="F67" s="4"/>
-      <c r="G67" s="4"/>
+      <c r="G67" s="5"/>
     </row>
     <row r="68" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C68" s="4" t="s">
@@ -1813,7 +1855,7 @@
       <c r="D68" s="4"/>
       <c r="E68" s="4"/>
       <c r="F68" s="4"/>
-      <c r="G68" s="4"/>
+      <c r="G68" s="5"/>
     </row>
     <row r="69" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C69" s="4" t="s">
@@ -1822,7 +1864,7 @@
       <c r="D69" s="4"/>
       <c r="E69" s="4"/>
       <c r="F69" s="4"/>
-      <c r="G69" s="4"/>
+      <c r="G69" s="5"/>
     </row>
     <row r="70" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C70" s="4" t="s">
@@ -1831,7 +1873,7 @@
       <c r="D70" s="4"/>
       <c r="E70" s="4"/>
       <c r="F70" s="4"/>
-      <c r="G70" s="4"/>
+      <c r="G70" s="5"/>
     </row>
     <row r="71" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C71" s="4" t="s">
@@ -1840,7 +1882,7 @@
       <c r="D71" s="4"/>
       <c r="E71" s="4"/>
       <c r="F71" s="4"/>
-      <c r="G71" s="4"/>
+      <c r="G71" s="5"/>
     </row>
     <row r="72" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C72" s="4" t="s">
@@ -1849,7 +1891,7 @@
       <c r="D72" s="4"/>
       <c r="E72" s="4"/>
       <c r="F72" s="4"/>
-      <c r="G72" s="4"/>
+      <c r="G72" s="5"/>
     </row>
     <row r="73" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C73" s="4" t="s">
@@ -1858,7 +1900,7 @@
       <c r="D73" s="4"/>
       <c r="E73" s="4"/>
       <c r="F73" s="4"/>
-      <c r="G73" s="4"/>
+      <c r="G73" s="5"/>
     </row>
     <row r="74" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C74" s="4" t="s">
@@ -1867,7 +1909,7 @@
       <c r="D74" s="4"/>
       <c r="E74" s="4"/>
       <c r="F74" s="4"/>
-      <c r="G74" s="4"/>
+      <c r="G74" s="5"/>
     </row>
     <row r="75" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C75" s="4" t="s">
@@ -1876,7 +1918,7 @@
       <c r="D75" s="4"/>
       <c r="E75" s="4"/>
       <c r="F75" s="4"/>
-      <c r="G75" s="4"/>
+      <c r="G75" s="5"/>
     </row>
     <row r="76" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C76" s="4" t="s">
@@ -1885,7 +1927,7 @@
       <c r="D76" s="4"/>
       <c r="E76" s="4"/>
       <c r="F76" s="4"/>
-      <c r="G76" s="4"/>
+      <c r="G76" s="5"/>
     </row>
     <row r="77" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C77" s="4" t="s">
@@ -1894,7 +1936,7 @@
       <c r="D77" s="4"/>
       <c r="E77" s="4"/>
       <c r="F77" s="4"/>
-      <c r="G77" s="4"/>
+      <c r="G77" s="5"/>
     </row>
     <row r="78" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C78" s="4" t="s">
@@ -1903,7 +1945,7 @@
       <c r="D78" s="4"/>
       <c r="E78" s="4"/>
       <c r="F78" s="4"/>
-      <c r="G78" s="4"/>
+      <c r="G78" s="5"/>
     </row>
     <row r="79" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C79" s="4" t="s">
@@ -1912,7 +1954,7 @@
       <c r="D79" s="4"/>
       <c r="E79" s="4"/>
       <c r="F79" s="4"/>
-      <c r="G79" s="4"/>
+      <c r="G79" s="5"/>
     </row>
     <row r="80" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C80" s="4" t="s">
@@ -1921,7 +1963,7 @@
       <c r="D80" s="4"/>
       <c r="E80" s="4"/>
       <c r="F80" s="4"/>
-      <c r="G80" s="4"/>
+      <c r="G80" s="5"/>
     </row>
     <row r="81" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C81" s="4" t="s">
@@ -1930,7 +1972,7 @@
       <c r="D81" s="4"/>
       <c r="E81" s="4"/>
       <c r="F81" s="4"/>
-      <c r="G81" s="4"/>
+      <c r="G81" s="5"/>
     </row>
     <row r="82" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C82" s="4" t="s">
@@ -1939,7 +1981,7 @@
       <c r="D82" s="4"/>
       <c r="E82" s="4"/>
       <c r="F82" s="4"/>
-      <c r="G82" s="4"/>
+      <c r="G82" s="5"/>
     </row>
     <row r="83" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C83" s="4" t="s">
@@ -1948,7 +1990,7 @@
       <c r="D83" s="4"/>
       <c r="E83" s="4"/>
       <c r="F83" s="4"/>
-      <c r="G83" s="4"/>
+      <c r="G83" s="5"/>
     </row>
     <row r="84" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C84" s="4" t="s">
@@ -1957,7 +1999,7 @@
       <c r="D84" s="4"/>
       <c r="E84" s="4"/>
       <c r="F84" s="4"/>
-      <c r="G84" s="4"/>
+      <c r="G84" s="5"/>
     </row>
     <row r="85" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C85" s="4" t="s">
@@ -1966,7 +2008,7 @@
       <c r="D85" s="4"/>
       <c r="E85" s="4"/>
       <c r="F85" s="4"/>
-      <c r="G85" s="4"/>
+      <c r="G85" s="5"/>
     </row>
     <row r="86" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C86" s="4" t="s">
@@ -1975,7 +2017,7 @@
       <c r="D86" s="4"/>
       <c r="E86" s="4"/>
       <c r="F86" s="4"/>
-      <c r="G86" s="4"/>
+      <c r="G86" s="5"/>
     </row>
     <row r="87" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C87" s="4" t="s">
@@ -1984,7 +2026,7 @@
       <c r="D87" s="4"/>
       <c r="E87" s="4"/>
       <c r="F87" s="4"/>
-      <c r="G87" s="4"/>
+      <c r="G87" s="5"/>
     </row>
     <row r="88" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C88" s="4" t="s">
@@ -1993,7 +2035,7 @@
       <c r="D88" s="4"/>
       <c r="E88" s="4"/>
       <c r="F88" s="4"/>
-      <c r="G88" s="4"/>
+      <c r="G88" s="5"/>
     </row>
     <row r="89" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C89" s="4" t="s">
@@ -2002,7 +2044,7 @@
       <c r="D89" s="4"/>
       <c r="E89" s="4"/>
       <c r="F89" s="4"/>
-      <c r="G89" s="4"/>
+      <c r="G89" s="5"/>
     </row>
     <row r="90" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C90" s="4" t="s">
@@ -2011,7 +2053,7 @@
       <c r="D90" s="4"/>
       <c r="E90" s="4"/>
       <c r="F90" s="4"/>
-      <c r="G90" s="4"/>
+      <c r="G90" s="5"/>
     </row>
     <row r="91" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C91" s="4" t="s">
@@ -2020,7 +2062,7 @@
       <c r="D91" s="4"/>
       <c r="E91" s="4"/>
       <c r="F91" s="4"/>
-      <c r="G91" s="4"/>
+      <c r="G91" s="5"/>
     </row>
     <row r="92" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C92" s="4" t="s">
@@ -2029,7 +2071,7 @@
       <c r="D92" s="4"/>
       <c r="E92" s="4"/>
       <c r="F92" s="4"/>
-      <c r="G92" s="4"/>
+      <c r="G92" s="5"/>
     </row>
     <row r="93" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C93" s="4" t="s">
@@ -2038,7 +2080,7 @@
       <c r="D93" s="4"/>
       <c r="E93" s="4"/>
       <c r="F93" s="4"/>
-      <c r="G93" s="4"/>
+      <c r="G93" s="5"/>
     </row>
     <row r="94" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C94" s="4" t="s">
@@ -2047,7 +2089,7 @@
       <c r="D94" s="4"/>
       <c r="E94" s="4"/>
       <c r="F94" s="4"/>
-      <c r="G94" s="4"/>
+      <c r="G94" s="5"/>
     </row>
     <row r="95" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C95" s="4" t="s">
@@ -2056,7 +2098,7 @@
       <c r="D95" s="4"/>
       <c r="E95" s="4"/>
       <c r="F95" s="4"/>
-      <c r="G95" s="4"/>
+      <c r="G95" s="5"/>
     </row>
     <row r="96" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C96" s="4" t="s">
@@ -2065,7 +2107,7 @@
       <c r="D96" s="4"/>
       <c r="E96" s="4"/>
       <c r="F96" s="4"/>
-      <c r="G96" s="4"/>
+      <c r="G96" s="5"/>
     </row>
     <row r="97" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C97" s="4" t="s">
@@ -2074,7 +2116,7 @@
       <c r="D97" s="4"/>
       <c r="E97" s="4"/>
       <c r="F97" s="4"/>
-      <c r="G97" s="4"/>
+      <c r="G97" s="5"/>
     </row>
     <row r="98" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C98" s="4" t="s">
@@ -2083,7 +2125,7 @@
       <c r="D98" s="4"/>
       <c r="E98" s="4"/>
       <c r="F98" s="4"/>
-      <c r="G98" s="4"/>
+      <c r="G98" s="5"/>
     </row>
     <row r="99" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C99" s="4" t="s">
@@ -2092,7 +2134,7 @@
       <c r="D99" s="4"/>
       <c r="E99" s="4"/>
       <c r="F99" s="4"/>
-      <c r="G99" s="4"/>
+      <c r="G99" s="5"/>
     </row>
     <row r="100" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C100" s="4" t="s">
@@ -2101,7 +2143,7 @@
       <c r="D100" s="4"/>
       <c r="E100" s="4"/>
       <c r="F100" s="4"/>
-      <c r="G100" s="4"/>
+      <c r="G100" s="5"/>
     </row>
     <row r="101" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C101" s="4" t="s">
@@ -2110,7 +2152,7 @@
       <c r="D101" s="4"/>
       <c r="E101" s="4"/>
       <c r="F101" s="4"/>
-      <c r="G101" s="4"/>
+      <c r="G101" s="5"/>
     </row>
     <row r="102" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C102" s="4" t="s">
@@ -2119,7 +2161,7 @@
       <c r="D102" s="4"/>
       <c r="E102" s="4"/>
       <c r="F102" s="4"/>
-      <c r="G102" s="4"/>
+      <c r="G102" s="5"/>
     </row>
     <row r="103" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C103" s="4" t="s">
@@ -2128,7 +2170,7 @@
       <c r="D103" s="4"/>
       <c r="E103" s="4"/>
       <c r="F103" s="4"/>
-      <c r="G103" s="4"/>
+      <c r="G103" s="5"/>
     </row>
     <row r="104" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C104" s="4" t="s">
@@ -2137,7 +2179,7 @@
       <c r="D104" s="4"/>
       <c r="E104" s="4"/>
       <c r="F104" s="4"/>
-      <c r="G104" s="4"/>
+      <c r="G104" s="5"/>
     </row>
     <row r="105" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C105" s="4" t="s">
@@ -2146,7 +2188,7 @@
       <c r="D105" s="4"/>
       <c r="E105" s="4"/>
       <c r="F105" s="4"/>
-      <c r="G105" s="4"/>
+      <c r="G105" s="5"/>
     </row>
     <row r="106" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C106" s="4" t="s">
@@ -2155,7 +2197,7 @@
       <c r="D106" s="4"/>
       <c r="E106" s="4"/>
       <c r="F106" s="4"/>
-      <c r="G106" s="4"/>
+      <c r="G106" s="5"/>
     </row>
     <row r="107" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C107" s="4" t="s">
@@ -2164,7 +2206,7 @@
       <c r="D107" s="4"/>
       <c r="E107" s="4"/>
       <c r="F107" s="4"/>
-      <c r="G107" s="4"/>
+      <c r="G107" s="5"/>
     </row>
     <row r="108" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C108" s="4" t="s">
@@ -2173,7 +2215,7 @@
       <c r="D108" s="4"/>
       <c r="E108" s="4"/>
       <c r="F108" s="4"/>
-      <c r="G108" s="4"/>
+      <c r="G108" s="5"/>
     </row>
     <row r="109" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C109" s="4" t="s">
@@ -2182,7 +2224,7 @@
       <c r="D109" s="4"/>
       <c r="E109" s="4"/>
       <c r="F109" s="4"/>
-      <c r="G109" s="4"/>
+      <c r="G109" s="5"/>
     </row>
     <row r="110" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C110" s="4" t="s">
@@ -2191,7 +2233,7 @@
       <c r="D110" s="4"/>
       <c r="E110" s="4"/>
       <c r="F110" s="4"/>
-      <c r="G110" s="4"/>
+      <c r="G110" s="5"/>
     </row>
     <row r="111" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C111" s="4" t="s">
@@ -2200,7 +2242,7 @@
       <c r="D111" s="4"/>
       <c r="E111" s="4"/>
       <c r="F111" s="4"/>
-      <c r="G111" s="4"/>
+      <c r="G111" s="5"/>
     </row>
     <row r="112" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C112" s="4" t="s">
@@ -2209,7 +2251,7 @@
       <c r="D112" s="4"/>
       <c r="E112" s="4"/>
       <c r="F112" s="4"/>
-      <c r="G112" s="4"/>
+      <c r="G112" s="5"/>
     </row>
     <row r="113" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C113" s="4" t="s">
@@ -2218,7 +2260,7 @@
       <c r="D113" s="4"/>
       <c r="E113" s="4"/>
       <c r="F113" s="4"/>
-      <c r="G113" s="4"/>
+      <c r="G113" s="5"/>
     </row>
     <row r="114" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C114" s="4" t="s">
@@ -2227,7 +2269,7 @@
       <c r="D114" s="4"/>
       <c r="E114" s="4"/>
       <c r="F114" s="4"/>
-      <c r="G114" s="4"/>
+      <c r="G114" s="5"/>
     </row>
     <row r="115" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C115" s="4" t="s">
@@ -2236,7 +2278,7 @@
       <c r="D115" s="4"/>
       <c r="E115" s="4"/>
       <c r="F115" s="4"/>
-      <c r="G115" s="4"/>
+      <c r="G115" s="5"/>
     </row>
     <row r="116" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C116" s="4" t="s">
@@ -2245,7 +2287,7 @@
       <c r="D116" s="4"/>
       <c r="E116" s="4"/>
       <c r="F116" s="4"/>
-      <c r="G116" s="4"/>
+      <c r="G116" s="5"/>
     </row>
     <row r="117" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C117" s="4" t="s">
@@ -2254,7 +2296,7 @@
       <c r="D117" s="4"/>
       <c r="E117" s="4"/>
       <c r="F117" s="4"/>
-      <c r="G117" s="4"/>
+      <c r="G117" s="5"/>
     </row>
     <row r="118" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C118" s="4" t="s">
@@ -2263,7 +2305,7 @@
       <c r="D118" s="4"/>
       <c r="E118" s="4"/>
       <c r="F118" s="4"/>
-      <c r="G118" s="4"/>
+      <c r="G118" s="5"/>
     </row>
     <row r="119" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C119" s="4" t="s">
@@ -2272,7 +2314,7 @@
       <c r="D119" s="4"/>
       <c r="E119" s="4"/>
       <c r="F119" s="4"/>
-      <c r="G119" s="4"/>
+      <c r="G119" s="5"/>
     </row>
     <row r="120" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C120" s="4" t="s">
@@ -2281,7 +2323,7 @@
       <c r="D120" s="4"/>
       <c r="E120" s="4"/>
       <c r="F120" s="4"/>
-      <c r="G120" s="4"/>
+      <c r="G120" s="5"/>
     </row>
     <row r="121" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C121" s="4" t="s">
@@ -2290,7 +2332,7 @@
       <c r="D121" s="4"/>
       <c r="E121" s="4"/>
       <c r="F121" s="4"/>
-      <c r="G121" s="4"/>
+      <c r="G121" s="5"/>
     </row>
     <row r="122" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C122" s="4" t="s">
@@ -2299,7 +2341,7 @@
       <c r="D122" s="4"/>
       <c r="E122" s="4"/>
       <c r="F122" s="4"/>
-      <c r="G122" s="4"/>
+      <c r="G122" s="5"/>
     </row>
     <row r="123" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C123" s="4" t="s">
@@ -2308,7 +2350,7 @@
       <c r="D123" s="4"/>
       <c r="E123" s="4"/>
       <c r="F123" s="4"/>
-      <c r="G123" s="4"/>
+      <c r="G123" s="5"/>
     </row>
     <row r="124" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C124" s="4" t="s">
@@ -2317,7 +2359,7 @@
       <c r="D124" s="4"/>
       <c r="E124" s="4"/>
       <c r="F124" s="4"/>
-      <c r="G124" s="4"/>
+      <c r="G124" s="5"/>
     </row>
     <row r="125" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C125" s="4" t="s">
@@ -2326,7 +2368,7 @@
       <c r="D125" s="4"/>
       <c r="E125" s="4"/>
       <c r="F125" s="4"/>
-      <c r="G125" s="4"/>
+      <c r="G125" s="5"/>
     </row>
     <row r="126" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C126" s="4" t="s">
@@ -2335,7 +2377,7 @@
       <c r="D126" s="4"/>
       <c r="E126" s="4"/>
       <c r="F126" s="4"/>
-      <c r="G126" s="4"/>
+      <c r="G126" s="5"/>
     </row>
     <row r="127" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C127" s="4" t="s">
@@ -2344,7 +2386,7 @@
       <c r="D127" s="4"/>
       <c r="E127" s="4"/>
       <c r="F127" s="4"/>
-      <c r="G127" s="4"/>
+      <c r="G127" s="5"/>
     </row>
     <row r="128" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C128" s="4" t="s">
@@ -2353,7 +2395,7 @@
       <c r="D128" s="4"/>
       <c r="E128" s="4"/>
       <c r="F128" s="4"/>
-      <c r="G128" s="4"/>
+      <c r="G128" s="5"/>
     </row>
     <row r="129" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C129" s="4" t="s">
@@ -2362,7 +2404,7 @@
       <c r="D129" s="4"/>
       <c r="E129" s="4"/>
       <c r="F129" s="4"/>
-      <c r="G129" s="4"/>
+      <c r="G129" s="5"/>
     </row>
     <row r="130" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C130" s="4" t="s">
@@ -2371,7 +2413,7 @@
       <c r="D130" s="4"/>
       <c r="E130" s="4"/>
       <c r="F130" s="4"/>
-      <c r="G130" s="4"/>
+      <c r="G130" s="5"/>
     </row>
     <row r="131" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C131" s="4" t="s">
@@ -2380,7 +2422,7 @@
       <c r="D131" s="4"/>
       <c r="E131" s="4"/>
       <c r="F131" s="4"/>
-      <c r="G131" s="4"/>
+      <c r="G131" s="5"/>
     </row>
     <row r="132" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C132" s="4" t="s">
@@ -2389,7 +2431,7 @@
       <c r="D132" s="4"/>
       <c r="E132" s="4"/>
       <c r="F132" s="4"/>
-      <c r="G132" s="4"/>
+      <c r="G132" s="5"/>
     </row>
     <row r="133" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C133" s="4" t="s">
@@ -2398,7 +2440,7 @@
       <c r="D133" s="4"/>
       <c r="E133" s="4"/>
       <c r="F133" s="4"/>
-      <c r="G133" s="4"/>
+      <c r="G133" s="5"/>
     </row>
     <row r="134" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C134" s="4" t="s">
@@ -2409,7 +2451,7 @@
         <v>211</v>
       </c>
       <c r="F134" s="4"/>
-      <c r="G134" s="4">
+      <c r="G134" s="5">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Se hicieron cambios en estos archivos
</commit_message>
<xml_diff>
--- a/Control.xlsx
+++ b/Control.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\10.106.12.32\compartir\openlayers2_nvo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{866FF221-E1A1-475E-887A-A3F8D7BEFA47}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BA7B973-1BF2-48CF-96EA-2B30DCCA15C7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="13905" xr2:uid="{119285BF-BAF3-43BB-BF3D-96AE8CA3F258}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="220">
   <si>
     <t>agregacgo.jsp</t>
   </si>
@@ -1515,19 +1515,27 @@
       <c r="C31" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D31" s="4"/>
-      <c r="E31" s="4"/>
+      <c r="D31" s="10"/>
+      <c r="E31" s="5" t="s">
+        <v>208</v>
+      </c>
       <c r="F31" s="4"/>
-      <c r="G31" s="5"/>
+      <c r="G31" s="5">
+        <v>2</v>
+      </c>
     </row>
     <row r="32" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C32" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D32" s="4"/>
-      <c r="E32" s="4"/>
+      <c r="D32" s="10"/>
+      <c r="E32" s="5" t="s">
+        <v>208</v>
+      </c>
       <c r="F32" s="4"/>
-      <c r="G32" s="5"/>
+      <c r="G32" s="5">
+        <v>2</v>
+      </c>
     </row>
     <row r="33" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C33" s="4" t="s">
@@ -1542,19 +1550,27 @@
       <c r="C34" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D34" s="4"/>
-      <c r="E34" s="4"/>
+      <c r="D34" s="10"/>
+      <c r="E34" s="5" t="s">
+        <v>208</v>
+      </c>
       <c r="F34" s="4"/>
-      <c r="G34" s="5"/>
+      <c r="G34" s="5">
+        <v>2</v>
+      </c>
     </row>
     <row r="35" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C35" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D35" s="4"/>
-      <c r="E35" s="4"/>
+      <c r="D35" s="10"/>
+      <c r="E35" s="5" t="s">
+        <v>208</v>
+      </c>
       <c r="F35" s="4"/>
-      <c r="G35" s="5"/>
+      <c r="G35" s="5">
+        <v>2</v>
+      </c>
     </row>
     <row r="36" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C36" s="4" t="s">

</xml_diff>

<commit_message>
Se corrigieron algunos archivos que tenian errores, y otros se cambio la consulta al archivo java.
</commit_message>
<xml_diff>
--- a/Control.xlsx
+++ b/Control.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\10.106.12.32\compartir\openlayers2_nvo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BA7B973-1BF2-48CF-96EA-2B30DCCA15C7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47A35444-8D2A-423D-8223-496919639C5A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="13905" xr2:uid="{119285BF-BAF3-43BB-BF3D-96AE8CA3F258}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="221">
   <si>
     <t>agregacgo.jsp</t>
   </si>
@@ -685,6 +685,9 @@
   </si>
   <si>
     <t>DESTINO</t>
+  </si>
+  <si>
+    <t>Se agrego una parte del codigo en el archivo java</t>
   </si>
 </sst>
 </file>
@@ -776,7 +779,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -803,6 +806,9 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="2" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1207,7 +1213,9 @@
       <c r="E7" s="5" t="s">
         <v>208</v>
       </c>
-      <c r="F7" s="7"/>
+      <c r="F7" s="7" t="s">
+        <v>220</v>
+      </c>
       <c r="G7" s="5">
         <v>1</v>
       </c>
@@ -1576,19 +1584,27 @@
       <c r="C36" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D36" s="4"/>
-      <c r="E36" s="4"/>
+      <c r="D36" s="10"/>
+      <c r="E36" s="13" t="s">
+        <v>208</v>
+      </c>
       <c r="F36" s="4"/>
-      <c r="G36" s="5"/>
+      <c r="G36" s="5">
+        <v>2</v>
+      </c>
     </row>
     <row r="37" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C37" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D37" s="4"/>
-      <c r="E37" s="4"/>
+      <c r="D37" s="10"/>
+      <c r="E37" s="13" t="s">
+        <v>208</v>
+      </c>
       <c r="F37" s="4"/>
-      <c r="G37" s="5"/>
+      <c r="G37" s="5">
+        <v>2</v>
+      </c>
     </row>
     <row r="38" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C38" s="4" t="s">
@@ -1607,28 +1623,40 @@
       <c r="C39" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D39" s="4"/>
-      <c r="E39" s="4"/>
-      <c r="F39" s="4"/>
-      <c r="G39" s="5"/>
+      <c r="D39" s="10"/>
+      <c r="E39" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="F39" s="5"/>
+      <c r="G39" s="5">
+        <v>2</v>
+      </c>
     </row>
     <row r="40" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C40" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D40" s="4"/>
-      <c r="E40" s="4"/>
+      <c r="D40" s="10"/>
+      <c r="E40" s="13" t="s">
+        <v>208</v>
+      </c>
       <c r="F40" s="4"/>
-      <c r="G40" s="5"/>
+      <c r="G40" s="5">
+        <v>2</v>
+      </c>
     </row>
     <row r="41" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C41" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D41" s="4"/>
-      <c r="E41" s="4"/>
+      <c r="D41" s="10"/>
+      <c r="E41" s="13" t="s">
+        <v>208</v>
+      </c>
       <c r="F41" s="4"/>
-      <c r="G41" s="5"/>
+      <c r="G41" s="5">
+        <v>2</v>
+      </c>
     </row>
     <row r="42" spans="3:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C42" s="4" t="s">

</xml_diff>